<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.002-02 Amir laisse le temps à Victorina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-02.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-02.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le canard sous la pluie</t>
+          <t>Amir laisse le temps à Victorina</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>entrée, pluie</t>
+          <t>classe, pupitre, fenêtre, sac, feuille, pull, bois, lumière, gomme</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Victorino, papa, maman</t>
+          <t>Amir, Victorina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Les manteaux gouttent. Victorino veut raconter le canard du fossé. Sarah connaît le mot. Elle attend. Il finit sa phrase.</t>
+          <t>La lumière pose un carré chaud sur le bois. Près du sac, un éclat de pupitre brille. Victorina cherche un mot. Amir le connaît, veut le dire maintenant, ouvre la bouche. Sourire parti. Il refuse de foncer, attend. Merci vécu. Deuxième ruse : un autre mot. Un éclat de pupitre tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les chaussures font un petit lac près de la porte. Les manteaux gouttent, goutte après goutte. Le radiateur fait tic-tic, tout doux. Dehors, la rue brille comme un miroir. Ça sent la laine mouillée. Posez les bottes sur le tapis, les enfants. Vous avez les pieds mouillés ? Un peu, maman. Je prends les écharpes. Elles sont froides encore. En ce moment, Sarah enlève son manteau près de Victorino. Un filet d'eau glisse le long d'une manche. Le tapis de l'entrée est rêche et gris. Je pose une serviette sous les bottes. La vitre est toute embuée, tu vois ? Oui. On dirait des rivières. Victorino a les joues roses. J'ai vu... Il s'arrête. Il cherche le mot. Sarah a vu le fossé, elle aussi. Elle sait le mot. Elle ouvre la bouche. On peut laisser le temps, Sarah. On attend la fin de la phrase. Sarah referme la bouche. Elle essuie une goutte sur sa manche. Elle compte tout bas. Un. Deux. Trois. Le radiateur tic-tac encore. J'ai vu un canard. Il avait le bec orange. Oui. Orange. Bravo, Sarah. Tu as su attendre. Maman tend deux chaussettes sèches. Enfilez ça. Doucement. Sarah s'assoit sur le bas de l'escalier. Le bois est un peu froid. Et après, il a... Victorino cherche encore. Sarah attend encore. Une goutte tombe du manteau, ploc. Il a fait coin-coin. Coin-coin, oui. Vous parlez l'un après l'autre. Sarah, tu as laissé le temps ? Oui, papa. On écoute jusqu'au bout. Plus tard, ils vont vers la cuisine. Le sol de l'entrée brille encore un peu. Demain, je veux... Sarah attend, les mains sur ses genoux. Demain je veux du pain pour les canards. Moi aussi. On en parlera demain, d'accord ? D'accord. Les manteaux sèchent près du radiateur. Ils sentent encore la pluie. On laisse les bottes ici. Elles font encore un petit lac. Oui. On attend qu'elles sèchent. Sarah a laissé le temps, encore une fois.</t>
+          <t>La lumière pose un carré chaud sur le bois. Ça sent le papier et la laine. Ça sent le pull, papa. Tu le sens, le bois, Amir ? Oui, papa. Un sac glisse contre un pupitre. Le tissu fait un bruit court. Il frotte, maman. Le sac tient près du bois ? Oui, maman. Près du sac, un éclat de pupitre brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La fenêtre tient un bout de ciel pâle. Il est clair, papa. Le ciel, là-bas ? Oui, là-bas. Victorina pose une feuille sur le bois. La feuille tremble entre ses doigts. Je connais le mot, maintenant ! Je le dis, tout de suite. Le mot de Victorina ? Oui. C'est facile. En ce moment, Amir se penche vers elle. Victorina ouvre la bouche. J'ai vu. Elle s'arrête. Elle cherche le mot. Amir a vu le canard, lui aussi. Il sait le mot. Il ouvre la bouche. Canard ! Le mot est sorti trop vite. Victorina baisse les yeux. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Tu vois Victorina, Amir ? Oui, papa. Ta bouche est ouverte, Amir ? Un peu, maman. L'éclat de pupitre tremble, puis tient. Victorina serre la feuille. Elle cherche, papa. Papa s'accroupit à la même hauteur. Amir regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les chaussures font un petit lac près de la porte. Les manteaux gouttent, goutte après goutte. Le radiateur fait tic-tic, tout doux. Dehors, la rue brille comme un miroir. Ça sent la laine mouillée. Posez les bottes sur le tapis, les enfants. Vous avez les pieds mouillés ? Un peu, maman. Je prends les écharpes. Elles sont froides encore. En ce moment, Sarah enlève son manteau près de Victorino. Un filet d'eau glisse le long d'une manche. Le tapis de l'entrée est rêche et gris. Je pose une serviette sous les bottes. La vitre est toute embuée, tu vois ? Oui. On dirait des rivières. Victorino a les joues roses. J'ai vu... Il s'arrête. Il cherche le mot. Sarah a vu le fossé, elle aussi. Elle sait le mot. Elle ouvre la bouche. On peut laisser le temps, Sarah. On attend la fin de la phrase. Sarah referme la bouche. Elle essuie une goutte sur sa manche. Elle compte tout bas. Un. Deux. Trois. Le radiateur tic-tac encore. J'ai vu un canard. Il avait le bec orange. Oui. Orange. Bravo, Sarah. Tu as su attendre. Maman tend deux chaussettes sèches. Enfilez ça. Doucement. Sarah s'assoit sur le bas de l'escalier. Le bois est un peu froid. Et après, il a... Victorino cherche encore. Sarah attend encore. Une goutte tombe du manteau, ploc. Il a fait coin-coin. Coin-coin, oui. Vous parlez l'un après l'autre. Sarah, tu as laissé le temps ? Oui, papa. On écoute jusqu'au bout. Plus tard, ils vont vers la cuisine. Le sol de l'entrée brille encore un peu. Demain, je veux... Sarah attend, les mains sur ses genoux. Demain je veux du pain pour les canards. Moi aussi. On en parlera demain, d'accord ? D'accord. Les manteaux sèchent près du radiateur. Ils sentent encore la pluie. On laisse les bottes ici. Elles font encore un petit lac. Oui. On attend qu'elles sèchent. Sarah a laissé le temps, encore une fois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La lumière pose un carré chaud sur le bois. Ça sent le papier et la laine. Ça sent le pull, papa. Tu le sens, le bois, Amir ? Oui, papa. Un sac glisse contre un pupitre. Le tissu fait un bruit court. Il frotte, maman. Le sac tient près du bois ? Oui, maman. Près du sac, un &lt;emphasis level="moderate"&gt;éclat de pupitre&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La fenêtre tient un bout de ciel pâle. Il est clair, papa. Le ciel, là-bas ? Oui, là-bas. Victorina pose une feuille sur le bois. La feuille tremble entre ses doigts. Je connais le mot, maintenant ! Je le dis, tout de suite. Le mot de Victorina ? Oui. C'est facile. En ce moment, Amir se penche vers elle. Victorina ouvre la bouche. J'ai vu. Elle s'arrête. Elle cherche le mot. Amir a vu le canard, lui aussi. Il sait le mot. Il ouvre la bouche. Canard ! Le mot est sorti trop vite. Victorina baisse les yeux. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Tu vois Victorina, Amir ? Oui, papa. Ta bouche est ouverte, Amir ? Un peu, maman. L'éclat de pupitre tremble, puis tient. Victorina serre la feuille. Elle cherche, papa. Papa s'accroupit à la même hauteur. Amir regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kenzo est en classe. Iris veut raconter son week-end. Elle dit : j'ai vu.. Puis elle cherche le mot. Kenzo connaît le mot. Il ouvre la bouche. La maîtresse dit : on peut &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. On n'achève pas à sa place. Kenzo attend la fin de la phrase. Iris respire. Elle dit : j'ai vu un canard. Kenzo sourit. Le soir, papa demande. Kenzo dit : j'ai su laisser le temps. [pause]</t>
+          <t>La lumière pose un carré chaud sur le bois. Ça sent le papier et la laine. Ça sent le pull, papa. Tu le sens, le bois, Amir ? Oui, papa. Un sac glisse contre un pupitre. Le tissu fait un bruit court. Il frotte, maman. Le sac tient près du bois ? Oui, maman. Près du sac, un &lt;emphasis&gt;éclat de pupitre&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La fenêtre tient un bout de ciel pâle. Il est clair, papa. Le ciel, là-bas ? Oui, là-bas. Victorina pose une feuille sur le bois. La feuille tremble entre ses doigts. Je connais le mot, maintenant ! Je le dis, tout de suite. Le mot de Victorina ? Oui. C'est facile. En ce moment, Amir se penche vers elle. Victorina ouvre la bouche. J'ai vu. Elle s'arrête. Elle cherche le mot. Amir a vu le canard, lui aussi. Il sait le mot. Il ouvre la bouche. Canard ! Le mot est sorti trop vite. Victorina baisse les yeux. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Tu vois Victorina, Amir ? Oui, papa. Ta bouche est ouverte, Amir ? Un peu, maman. L'éclat de pupitre tremble, puis tient. Victorina serre la feuille. Elle cherche, papa. Papa s'accroupit à la même hauteur. Amir regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>éclat de pupitre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,78 +1321,67 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_dire_le_mot_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les chaussures font un petit lac près de la porte.
-narrateur|Les manteaux gouttent, goutte après goutte.
-narrateur|Le radiateur fait tic-tic, tout doux.
-narrateur|Dehors, la rue brille comme un miroir.
-narrateur|Ça sent la laine mouillée.
-maman|Posez les bottes sur le tapis, les enfants.
-maman|Vous avez les pieds mouillés ?
-enfant-f|Un peu, maman.
-papa|Je prends les écharpes.
-papa|Elles sont froides encore.
-narrateur|En ce moment, Sarah enlève son manteau près de Victorino.
-narrateur|Un filet d'eau glisse le long d'une manche.
-narrateur|Le tapis de l'entrée est rêche et gris.
-maman|Je pose une serviette sous les bottes.
-papa|La vitre est toute embuée, tu vois ?
-enfant-f|Oui.
-enfant-f|On dirait des rivières.
-narrateur|Victorino a les joues roses.
-copain|J'ai vu...
-narrateur|Il s'arrête.
-narrateur|Il cherche le mot.
-narrateur|Sarah a vu le fossé, elle aussi.
-narrateur|Elle sait le mot.
-narrateur|Elle ouvre la bouche.
-papa|On peut laisser le temps, Sarah.
-papa|On attend la fin de la phrase.
-narrateur|Sarah referme la bouche.
-narrateur|Elle essuie une goutte sur sa manche.
-narrateur|Elle compte tout bas.
-narrateur|Un.
-narrateur|Deux.
-narrateur|Trois.
-narrateur|Le radiateur tic-tac encore.
-copain|J'ai vu un canard.
-enfant-f|Il avait le bec orange.
-copain|Oui.
-copain|Orange.
-maman|Bravo, Sarah.
-maman|Tu as su attendre.
-narrateur|Maman tend deux chaussettes sèches.
-maman|Enfilez ça.
-maman|Doucement.
-narrateur|Sarah s'assoit sur le bas de l'escalier.
-narrateur|Le bois est un peu froid.
-copain|Et après, il a...
-narrateur|Victorino cherche encore.
-narrateur|Sarah attend encore.
-narrateur|Une goutte tombe du manteau, ploc.
-copain|Il a fait coin-coin.
-enfant-f|Coin-coin, oui.
-papa|Vous parlez l'un après l'autre.
-papa|Sarah, tu as laissé le temps ?
-enfant-f|Oui, papa.
-papa|On écoute jusqu'au bout.
-narrateur|Plus tard, ils vont vers la cuisine.
-narrateur|Le sol de l'entrée brille encore un peu.
-copain|Demain, je veux...
-narrateur|Sarah attend, les mains sur ses genoux.
-copain|Demain je veux du pain pour les canards.
-enfant-f|Moi aussi.
-maman|On en parlera demain, d'accord ?
-copain|D'accord.
-narrateur|Les manteaux sèchent près du radiateur.
-narrateur|Ils sentent encore la pluie.
-papa|On laisse les bottes ici.
-enfant-f|Elles font encore un petit lac.
-maman|Oui.
-maman|On attend qu'elles sèchent.
-narrateur|Sarah a laissé le temps, encore une fois.</t>
+          <t>narrateur|La lumière pose un carré chaud sur le bois.
+narrateur|Ça sent le papier et la laine.
+enfant-m|Ça sent le pull, papa.
+papa|Tu le sens, le bois, Amir ?
+enfant-m|Oui, papa.
+narrateur|Un sac glisse contre un pupitre.
+narrateur|Le tissu fait un bruit court.
+enfant-m|Il frotte, maman.
+maman|Le sac tient près du bois ?
+enfant-m|Oui, maman.
+narrateur|Près du sac, un éclat de pupitre brille.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|La fenêtre tient un bout de ciel pâle.
+enfant-m|Il est clair, papa.
+papa|Le ciel, là-bas ?
+enfant-m|Oui, là-bas.
+narrateur|Victorina pose une feuille sur le bois.
+narrateur|La feuille tremble entre ses doigts.
+enfant-m|Je connais le mot, maintenant !
+enfant-m|Je le dis, tout de suite.
+papa|Le mot de Victorina ?
+enfant-m|Oui.
+enfant-m|C'est facile.
+narrateur|En ce moment, Amir se penche vers elle.
+narrateur|Victorina ouvre la bouche.
+copine|J'ai vu.
+narrateur|Elle s'arrête.
+narrateur|Elle cherche le mot.
+narrateur|Amir a vu le canard, lui aussi.
+narrateur|Il sait le mot.
+narrateur|Il ouvre la bouche.
+enfant-m|Canard !
+narrateur|Le mot est sorti trop vite.
+narrateur|Victorina baisse les yeux.
+enfant-m|Oh.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+papa|Tu vois Victorina, Amir ?
+enfant-m|Oui, papa.
+maman|Ta bouche est ouverte, Amir ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de pupitre tremble, puis tient.
+narrateur|Victorina serre la feuille.
+enfant-m|Elle cherche, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Amir regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>classe</t>
         </is>
       </c>
     </row>
@@ -1419,17 +1408,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorino cherche un mot. Que fait Sarah ?</t>
+          <t>Victorina cherche un mot. Que fait Amir ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino cherche un mot. Que fait Sarah ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina cherche un mot. Que fait &lt;emphasis level="moderate"&gt;Amir&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Iris cherche un mot. Que fait Kenzo ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina cherche un mot. Que fait &lt;emphasis&gt;Amir&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1454,7 +1443,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On n'achève pas à sa place. Que fait Kenzo ?</t>
+          <t>On n'achève pas à sa place. Que fait Amir ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1492,18 +1481,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1518,34 +1507,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Amir</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1554,29 +1547,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=victorina_cherche_un_mot_que_fait_amir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorino cherche un mot.
-narrateur|Que fait Sarah ?</t>
+          <t>narrateur|Victorina cherche un mot.
+narrateur|Que fait Amir ?</t>
         </is>
       </c>
     </row>
@@ -1603,17 +1596,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a su laisser le temps. Victorino a fini sa phrase. On attend la fin de la phrase. Bravo, Sarah. J'ai laissé le temps. Le canard a eu tout son récit.</t>
+          <t>Amir connaît le mot. Je le dis, maintenant ! Il avance trop vite vers le mot. Les mots se bousculent dans sa bouche. Victorina baisse les yeux. Elle serre la feuille contre elle. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la feuille, un instant. Il écoute le silence de la classe. Tu restes près d'elle, Amir ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Amir reste un moment, les mains ouvertes. Il attend. Victorina souffle. J'ai vu un canard. Le canard. Oui. Merci, Amir. Papa a vu les deux, près du pupitre. Le papier est tiède, sous les doigts. Il est chaud. Victorina glisse la main sur le dessin. Le canard. Il a un bec, là ? Oui, là. Amir pose les mains sur le bois. Il reste, sans se presser. Tes mains sont au chaud, Amir ? Un peu, maman. Victorina s'assoit plus droit. Orange. Orange, oui. La feuille tient sur le pupitre ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a su laisser le temps. Victorino a fini sa phrase. On attend la fin de la phrase. Bravo, Sarah. J'ai laissé le temps. Le canard a eu tout son récit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir connaît le mot. Je le dis, maintenant ! Il avance trop vite vers le mot. Les mots se bousculent dans sa bouche. Victorina baisse les yeux. Elle serre la feuille contre elle. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la feuille, un instant. Il écoute le silence de la classe. Tu restes près d'elle, Amir ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Amir reste un moment, les mains ouvertes. Il attend. Victorina souffle. J'ai vu un &lt;emphasis level="moderate"&gt;canard&lt;/emphasis&gt;. Le canard. Oui. Merci, Amir. Papa a vu les deux, près du pupitre. Le papier est tiède, sous les doigts. Il est chaud. Victorina glisse la main sur le dessin. Le canard. Il a un bec, là ? Oui, là. Amir pose les mains sur le bois. Il reste, sans se presser. Tes mains sont au chaud, Amir ? Un peu, maman. Victorina s'assoit plus droit. Orange. Orange, oui. La feuille tient sur le pupitre ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Kenzo a su &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. Iris a fini sa phrase. [pause]</t>
+          <t>Amir connaît le mot. Je le dis, maintenant ! Il avance trop vite vers le mot. Les mots se bousculent dans sa bouche. Victorina baisse les yeux. Elle serre la feuille contre elle. Oh. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la feuille, un instant. Il écoute le silence de la classe. Tu restes près d'elle, Amir ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Amir reste un moment, les mains ouvertes. Il attend. Victorina souffle. J'ai vu un &lt;emphasis&gt;canard&lt;/emphasis&gt;. Le canard. Oui. Merci, Amir. Papa a vu les deux, près du pupitre. Le papier est tiède, sous les doigts. Il est chaud. Victorina glisse la main sur le dessin. Le canard. Il a un bec, là ? Oui, là. Amir pose les mains sur le bois. Il reste, sans se presser. Tes mains sont au chaud, Amir ? Un peu, maman. Victorina s'assoit plus droit. Orange. Orange, oui. La feuille tient sur le pupitre ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1660,7 +1653,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1668,10 +1661,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1694,30 +1687,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>canard</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1726,10 +1719,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1742,17 +1735,57 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah a su laisser le temps.
-narrateur|Victorino a fini sa phrase.
-papa|On attend la fin de la phrase.
-maman|Bravo, Sarah.
-enfant-f|J'ai laissé le temps.
-papa|Le canard a eu tout son récit.</t>
+          <t>narrateur|Amir connaît le mot.
+enfant-m|Je le dis, maintenant !
+narrateur|Il avance trop vite vers le mot.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Victorina baisse les yeux.
+narrateur|Elle serre la feuille contre elle.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la feuille, un instant.
+narrateur|Il écoute le silence de la classe.
+papa|Tu restes près d'elle, Amir ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Papa, on fait quoi ?
+papa|On pose les mains, puis on reste.
+enfant-m|D'accord.
+narrateur|Amir reste un moment, les mains ouvertes.
+narrateur|Il attend.
+narrateur|Victorina souffle.
+copine|J'ai vu un canard.
+enfant-m|Le canard.
+copine|Oui.
+papa|Merci, Amir.
+narrateur|Papa a vu les deux, près du pupitre.
+maman|Le papier est tiède, sous les doigts.
+enfant-m|Il est chaud.
+narrateur|Victorina glisse la main sur le dessin.
+enfant-m|Le canard.
+papa|Il a un bec, là ?
+enfant-m|Oui, là.
+narrateur|Amir pose les mains sur le bois.
+narrateur|Il reste, sans se presser.
+maman|Tes mains sont au chaud, Amir ?
+enfant-m|Un peu, maman.
+narrateur|Victorina s'assoit plus droit.
+copine|Orange.
+enfant-m|Orange, oui.
+maman|La feuille tient sur le pupitre ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>feuille</t>
         </is>
       </c>
     </row>
@@ -1779,17 +1812,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa serre la main de Sarah. Tes chaussettes sont sèches, maintenant ? Oui, papa. On rentre dans le salon, tout doucement. Les bottes restent près de la porte. Le petit lac a disparu. Dehors, la pluie est plus fine.</t>
+          <t>Ils restent près du pupitre. Victorina reprend la feuille. Et après, il a. Elle cherche. La suite, maintenant ! Amir ouvre la bouche trop vite. Le mot pousse contre les dents. Amir avance les lèvres, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Sa bouche se ferme, puis s'ouvre sans bruit. Personne ne dit la suite. Il observe la feuille, un instant. Il écoute le silence du pupitre. Au bord du bois, un éclat de pupitre luit. Là, sur le bois. Tu dis la suite, Victorina ? Victorina ne dit rien, d'abord. Elle tient la feuille, sans parler. Il a fait coin-coin. Amir hoche la tête, sans se presser. Victorina souffle, plus lentement. Le papier est lisse et tiède. Tu l'entends, le canard ? Oui, papa. La feuille est près du sac ? Oui, maman. Une gomme roule vers le bord. Amir pose une main dessus. Victorina pose la suivante. La gomme tient, Amir ? Oui, papa. Un rayon passe sur le pupitre. Il allume le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa serre la main de Sarah. Tes chaussettes sont sèches, maintenant ? Oui, papa. On rentre dans le salon, tout doucement. Les bottes restent près de la porte. Le petit lac a disparu. Dehors, la pluie est plus fine.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près du pupitre. Victorina reprend la feuille. Et après, il a. Elle cherche. La suite, maintenant ! Amir ouvre la bouche trop vite. Le mot pousse contre les dents. Amir avance les lèvres, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Sa bouche se ferme, puis s'ouvre sans bruit. Personne ne dit la suite. Il observe la feuille, un instant. Il écoute le silence du pupitre. Au bord du bois, un &lt;emphasis level="moderate"&gt;éclat de pupitre&lt;/emphasis&gt; luit. Là, sur le bois. Tu dis la suite, Victorina ? Victorina ne dit rien, d'abord. Elle tient la feuille, sans parler. Il a fait coin-coin. Amir hoche la tête, sans se presser. Victorina souffle, plus lentement. Le papier est lisse et tiède. Tu l'entends, le canard ? Oui, papa. La feuille est près du sac ? Oui, maman. Une gomme roule vers le bord. Amir pose une main dessus. Victorina pose la suivante. La gomme tient, Amir ? Oui, papa. Un rayon passe sur le pupitre. Il allume le bois.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa serre la &lt;emphasis&gt;main&lt;/emphasis&gt; de Kenzo. Ils rentrent. [pause]</t>
+          <t>Ils restent près du pupitre. Victorina reprend la feuille. Et après, il a. Elle cherche. La suite, maintenant ! Amir ouvre la bouche trop vite. Le mot pousse contre les dents. Amir avance les lèvres, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Sa bouche se ferme, puis s'ouvre sans bruit. Personne ne dit la suite. Il observe la feuille, un instant. Il écoute le silence du pupitre. Au bord du bois, un &lt;emphasis&gt;éclat de pupitre&lt;/emphasis&gt; luit. Là, sur le bois. Tu dis la suite, Victorina ? Victorina ne dit rien, d'abord. Elle tient la feuille, sans parler. Il a fait coin-coin. Amir hoche la tête, sans se presser. Victorina souffle, plus lentement. Le papier est lisse et tiède. Tu l'entends, le canard ? Oui, papa. La feuille est près du sac ? Oui, maman. Une gomme roule vers le bord. Amir pose une main dessus. Victorina pose la suivante. La gomme tient, Amir ? Oui, papa. Un rayon passe sur le pupitre. Il allume le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1836,7 +1869,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1844,10 +1877,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1870,30 +1903,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de pupitre</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1902,10 +1935,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1916,16 +1949,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=autre_mot_trop_vite_il_attend; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa serre la main de Sarah.
-papa|Tes chaussettes sont sèches, maintenant ?
-enfant-f|Oui, papa.
-maman|On rentre dans le salon, tout doucement.
-narrateur|Les bottes restent près de la porte.
-narrateur|Le petit lac a disparu.
-narrateur|Dehors, la pluie est plus fine.</t>
+          <t>narrateur|Ils restent près du pupitre.
+narrateur|Victorina reprend la feuille.
+copine|Et après, il a.
+narrateur|Elle cherche.
+enfant-m|La suite, maintenant !
+narrateur|Amir ouvre la bouche trop vite.
+narrateur|Le mot pousse contre les dents.
+narrateur|Amir avance les lèvres, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Sa bouche se ferme, puis s'ouvre sans bruit.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la feuille, un instant.
+narrateur|Il écoute le silence du pupitre.
+narrateur|Au bord du bois, un éclat de pupitre luit.
+enfant-m|Là, sur le bois.
+enfant-m|Tu dis la suite, Victorina ?
+narrateur|Victorina ne dit rien, d'abord.
+narrateur|Elle tient la feuille, sans parler.
+copine|Il a fait coin-coin.
+narrateur|Amir hoche la tête, sans se presser.
+narrateur|Victorina souffle, plus lentement.
+narrateur|Le papier est lisse et tiède.
+papa|Tu l'entends, le canard ?
+enfant-m|Oui, papa.
+maman|La feuille est près du sac ?
+enfant-m|Oui, maman.
+narrateur|Une gomme roule vers le bord.
+narrateur|Amir pose une main dessus.
+narrateur|Victorina pose la suivante.
+papa|La gomme tient, Amir ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le pupitre.
+enfant-m|Il allume le bois.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>sac</t>
         </is>
       </c>
     </row>
@@ -1952,17 +2021,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Le manteau de Victorino sèche encore.</t>
+          <t>Ils restent près du pupitre. Le canard a eu sa phrase, Amir ? Oui, maman. Tu souffles un peu ? Oui, papa. Amir souffle, un filet d'air. Le papier sent bon. Tu le sens, le dessin ? Oui, maman. La feuille reste un peu, à plat. Elle a tenu, sur le bois. Canard. Le pupitre est chaud, sous les mains. La feuille fait une petite ombre. On y revient, après. Un éclat de pupitre tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Le manteau de Victorino sèche encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du pupitre. Le canard a eu sa phrase, Amir ? Oui, maman. Tu souffles un peu ? Oui, papa. Amir souffle, un filet d'air. Le papier sent bon. Tu le sens, le dessin ? Oui, maman. La feuille reste un peu, à plat. Elle a tenu, sur le bois. Canard. Le pupitre est chaud, sous les mains. La feuille fait une petite ombre. On y revient, après. Un &lt;emphasis level="moderate"&gt;éclat de pupitre&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du pupitre. Le canard a eu sa phrase, Amir ? Oui, maman. Tu souffles un peu ? Oui, papa. Amir souffle, un filet d'air. Le papier sent bon. Tu le sens, le dessin ? Oui, maman. La feuille reste un peu, à plat. Elle a tenu, sur le bois. Canard. Le pupitre est chaud, sous les mains. La feuille fait une petite ombre. On y revient, après. Un &lt;emphasis&gt;éclat de pupitre&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2009,18 +2078,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2029,12 +2098,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2043,17 +2112,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pupitre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2062,11 +2135,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2075,26 +2148,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai attendu la fin.
-papa|Bravo.
-narrateur|Le manteau de Victorino sèche encore.</t>
+          <t>narrateur|Ils restent près du pupitre.
+maman|Le canard a eu sa phrase, Amir ?
+enfant-m|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-m|Oui, papa.
+narrateur|Amir souffle, un filet d'air.
+enfant-m|Le papier sent bon.
+maman|Tu le sens, le dessin ?
+enfant-m|Oui, maman.
+papa|La feuille reste un peu, à plat.
+enfant-m|Elle a tenu, sur le bois.
+copine|Canard.
+narrateur|Le pupitre est chaud, sous les mains.
+narrateur|La feuille fait une petite ombre.
+enfant-m|On y revient, après.
+narrateur|Un éclat de pupitre tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2179,6 +2269,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>